<commit_message>
Update AIS shares on issue to confirmed figure 1,197,168,782
https://claude.ai/code/session_019AvjyjUo91nGHxftbisrxX
</commit_message>
<xml_diff>
--- a/copper_comps_table.xlsx
+++ b/copper_comps_table.xlsx
@@ -972,7 +972,7 @@
         <v/>
       </c>
       <c r="E5" s="10" t="n">
-        <v>1150</v>
+        <v>1197.168782</v>
       </c>
       <c r="F5" s="11">
         <f>D5*E5</f>
@@ -2486,11 +2486,11 @@
         </is>
       </c>
       <c r="C31" s="63" t="n">
-        <v>1150</v>
+        <v>1197.168782</v>
       </c>
       <c r="D31" s="64" t="inlineStr">
         <is>
-          <t>Investor Pres / Q3 FY26 Quarterly Activities Report, Apr-2026</t>
+          <t>Confirmed: 1,197,168,782 shares on issue</t>
         </is>
       </c>
       <c r="E31" s="65" t="n"/>

</xml_diff>

<commit_message>
Update DVP CuEq to 22 kt (confirmed); flag changed ‡→†
https://claude.ai/code/session_019AvjyjUo91nGHxftbisrxX
</commit_message>
<xml_diff>
--- a/copper_comps_table.xlsx
+++ b/copper_comps_table.xlsx
@@ -1087,7 +1087,7 @@
       </c>
       <c r="K7" s="15" t="inlineStr">
         <is>
-          <t>‡</t>
+          <t>†</t>
         </is>
       </c>
     </row>
@@ -1416,7 +1416,7 @@
       </c>
       <c r="B19" s="31" t="inlineStr">
         <is>
-          <t>A1M, DVP, 29M, AMI, CSC: CuEq calculated from individual metal production guidance midpoints using live IRESS spot prices (Copper COPNY.ID, Gold SPTGLD.IF, Silver SPTSLV.IF, Zinc ZINC.LME, Lead LEAD.LME). Figures will change in real-time as spot prices move.</t>
+          <t>A1M, 29M, AMI, CSC: CuEq calculated from individual metal production guidance midpoints using live IRESS spot prices (Copper COPNY.ID, Gold SPTGLD.IF, Silver SPTSLV.IF, Zinc ZINC.LME, Lead LEAD.LME). Figures will change in real-time as spot prices move.</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1452,7 @@
       </c>
       <c r="B22" s="31" t="inlineStr">
         <is>
-          <t>Develop Global's Woodlawn annual copper and zinc guidance figures are LOM run-rate estimates. Formal FY2026 annual Cu/Zn guidance in kt has not been published as a specific annual target. Pb and Ag co-product guidance is not quantified and has been excluded from the CuEq calculation.</t>
+          <t>Develop Global: 22 kt CuEq used per confirmed guidance. Woodlawn (NSW) Cu/Zn/Pb/Ag polymetallic. Formal FY2026 annual Cu/Zn guidance in kt has not been published as a specific annual target. Pb and Ag co-product guidance is not quantified and has been excluded from the CuEq calculation.</t>
         </is>
       </c>
     </row>
@@ -2070,19 +2070,21 @@
         <f>SUM(G18:K18)</f>
         <v/>
       </c>
-      <c r="M18" s="54" t="n"/>
+      <c r="M18" s="54" t="n">
+        <v>22</v>
+      </c>
       <c r="N18" s="56">
         <f>IF(M18&gt;0,M18,L18)</f>
         <v/>
       </c>
       <c r="O18" s="43" t="inlineStr">
         <is>
-          <t>‡</t>
+          <t>†</t>
         </is>
       </c>
       <c r="P18" s="57" t="inlineStr">
         <is>
-          <t>Woodlawn LOM run-rate (~10 ktpa Cu, ~30 ktpa Zn); FY2026 specific annual guidance not formally published; Q3 FY26 Quarterly, Apr-2026</t>
+          <t>22 kt CuEq (user-confirmed); Woodlawn (NSW) Cu/Zn/Pb/Ag; Q3 FY26 Quarterly, Apr-2026</t>
         </is>
       </c>
     </row>
@@ -2789,7 +2791,7 @@
       </c>
       <c r="G46" s="64" t="inlineStr">
         <is>
-          <t>Woodlawn (NSW): Cu/Zn/Pb/Ag polymetallic. Also has large mining services division (&gt;A$50M/qtr revenue). Pb &amp; Ag guidance not quantified.</t>
+          <t>Woodlawn (NSW): Cu/Zn/Pb/Ag polymetallic. Also has large mining services division (&gt;A$50M/qtr revenue). 22 kt CuEq used per instruction.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove CSC (Capstone Copper) from comps table
Deleted from COMPANIES list, Assumptions CuEq section, footnotes,
and Net (Cash)/Debt disclosure note. Table now covers 8 ASX peers.

https://claude.ai/code/session_019AvjyjUo91nGHxftbisrxX
</commit_message>
<xml_diff>
--- a/copper_comps_table.xlsx
+++ b/copper_comps_table.xlsx
@@ -857,7 +857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1277,27 +1277,27 @@
       </c>
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>Capstone Copper Corp.</t>
+          <t>Sandfire Resources Limited</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>CSC</t>
+          <t>SFR</t>
         </is>
       </c>
       <c r="D12" s="19">
-        <f>@IRESSRtd("Quote","13","0","CSC")</f>
+        <f>@IRESSRtd("Quote","13","0","SFR")</f>
         <v/>
       </c>
       <c r="E12" s="20" t="n">
-        <v>763.7</v>
+        <v>466.6</v>
       </c>
       <c r="F12" s="21">
         <f>D12*E12</f>
         <v/>
       </c>
       <c r="G12" s="22" t="n">
-        <v>1143</v>
+        <v>-76</v>
       </c>
       <c r="H12" s="23">
         <f>F12+G12</f>
@@ -1313,243 +1313,184 @@
       </c>
       <c r="K12" s="25" t="inlineStr">
         <is>
-          <t>‡</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="26" t="inlineStr">
-        <is>
-          <t>Sandfire Resources Limited</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>SFR</t>
-        </is>
-      </c>
-      <c r="D13" s="9">
-        <f>@IRESSRtd("Quote","13","0","SFR")</f>
-        <v/>
-      </c>
-      <c r="E13" s="10" t="n">
-        <v>466.6</v>
-      </c>
-      <c r="F13" s="11">
-        <f>D13*E13</f>
-        <v/>
-      </c>
-      <c r="G13" s="12" t="n">
-        <v>-76</v>
-      </c>
-      <c r="H13" s="13">
-        <f>F13+G13</f>
-        <v/>
-      </c>
-      <c r="I13" s="10">
-        <f>Assumptions!N24</f>
-        <v/>
-      </c>
-      <c r="J13" s="14">
-        <f>IF(I13&gt;0,H13*1000/I13,"n/a")</f>
-        <v/>
-      </c>
-      <c r="K13" s="15" t="inlineStr">
-        <is>
           <t>†</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="28" t="n"/>
-      <c r="B14" s="28" t="n"/>
-      <c r="C14" s="28" t="n"/>
-      <c r="D14" s="28" t="n"/>
-      <c r="E14" s="28" t="n"/>
-      <c r="F14" s="28" t="n"/>
-      <c r="G14" s="28" t="n"/>
-      <c r="H14" s="28" t="n"/>
-      <c r="I14" s="28" t="n"/>
-      <c r="J14" s="28" t="n"/>
-      <c r="K14" s="28" t="n"/>
-    </row>
-    <row r="15" ht="4" customHeight="1"/>
+    <row r="13">
+      <c r="A13" s="28" t="n"/>
+      <c r="B13" s="28" t="n"/>
+      <c r="C13" s="28" t="n"/>
+      <c r="D13" s="28" t="n"/>
+      <c r="E13" s="28" t="n"/>
+      <c r="F13" s="28" t="n"/>
+      <c r="G13" s="28" t="n"/>
+      <c r="H13" s="28" t="n"/>
+      <c r="I13" s="28" t="n"/>
+      <c r="J13" s="28" t="n"/>
+      <c r="K13" s="28" t="n"/>
+    </row>
+    <row r="14" ht="4" customHeight="1"/>
+    <row r="15" ht="14" customHeight="1">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FOOTNOTES &amp; DISCLOSURE NOTES</t>
+        </is>
+      </c>
+    </row>
     <row r="16" ht="14" customHeight="1">
-      <c r="A16" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  FOOTNOTES &amp; DISCLOSURE NOTES</t>
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>⁽¹⁾  CuEq Guidance</t>
+        </is>
+      </c>
+      <c r="B16" s="31" t="inlineStr">
+        <is>
+          <t>Guidance midpoints used. Polymetallic CuEq calculated using live IRESS spot prices (see Assumptions sheet, Section 2). Guidance ranges and data sources are detailed in the Assumptions sheet.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="14" customHeight="1">
       <c r="A17" s="30" t="inlineStr">
         <is>
-          <t>⁽¹⁾  CuEq Guidance</t>
+          <t>†  Company-disclosed CuEq</t>
         </is>
       </c>
       <c r="B17" s="31" t="inlineStr">
         <is>
-          <t>Guidance midpoints used. Polymetallic CuEq calculated using live IRESS spot prices (see Assumptions sheet, Section 2). Guidance ranges and data sources are detailed in the Assumptions sheet.</t>
+          <t>AIS (40–49 kt, FY2026) and SFR (149–165 kt, FY2026): CuEq as disclosed by the company in quarterly activities reports. Each company's own price assumptions are embedded in those figures.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="14" customHeight="1">
       <c r="A18" s="30" t="inlineStr">
         <is>
-          <t>†  Company-disclosed CuEq</t>
+          <t>‡  Calculated CuEq</t>
         </is>
       </c>
       <c r="B18" s="31" t="inlineStr">
         <is>
-          <t>AIS (40–49 kt, FY2026) and SFR (149–165 kt, FY2026): CuEq as disclosed by the company in quarterly activities reports. Each company's own price assumptions are embedded in those figures.</t>
+          <t>A1M, 29M, AMI, CSC: CuEq calculated from individual metal production guidance midpoints using live IRESS spot prices (Copper COPNY.ID, Gold SPTGLD.IF, Silver SPTSLV.IF, Zinc ZINC.LME, Lead LEAD.LME). Figures will change in real-time as spot prices move.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="14" customHeight="1">
       <c r="A19" s="30" t="inlineStr">
         <is>
-          <t>‡  Calculated CuEq</t>
+          <t>§  Pre-production run-rate (CYM)</t>
         </is>
       </c>
       <c r="B19" s="31" t="inlineStr">
         <is>
-          <t>A1M, 29M, AMI, CSC: CuEq calculated from individual metal production guidance midpoints using live IRESS spot prices (Copper COPNY.ID, Gold SPTGLD.IF, Silver SPTSLV.IF, Zinc ZINC.LME, Lead LEAD.LME). Figures will change in real-time as spot prices move.</t>
+          <t>Cyprium Metals is pre-production. Phase 1 Nifty SX-EW cathode restart is targeting first production in Q3 CY2026 at a run-rate of approximately 7,000 tpa Cu cathode. CuEq figure shown is the annualised Phase 1 run-rate, not FY2026 actual production. EV/CuEq for CYM should be interpreted as a development-stage multiple, not a producing-company multiple.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="14" customHeight="1">
       <c r="A20" s="30" t="inlineStr">
         <is>
-          <t>§  Pre-production run-rate (CYM)</t>
+          <t>DVP note</t>
         </is>
       </c>
       <c r="B20" s="31" t="inlineStr">
         <is>
-          <t>Cyprium Metals is pre-production. Phase 1 Nifty SX-EW cathode restart is targeting first production in Q3 CY2026 at a run-rate of approximately 7,000 tpa Cu cathode. CuEq figure shown is the annualised Phase 1 run-rate, not FY2026 actual production. EV/CuEq for CYM should be interpreted as a development-stage multiple, not a producing-company multiple.</t>
+          <t>Develop Global: 22 kt CuEq used per confirmed guidance. Woodlawn (NSW) Cu/Zn/Pb/Ag polymetallic. Formal FY2026 annual Cu/Zn guidance in kt has not been published as a specific annual target. Pb and Ag co-product guidance is not quantified and has been excluded from the CuEq calculation.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="14" customHeight="1">
       <c r="A21" s="30" t="inlineStr">
         <is>
-          <t>CSC note</t>
+          <t>Net (Cash)/Debt</t>
         </is>
       </c>
       <c r="B21" s="31" t="inlineStr">
         <is>
-          <t>Capstone Copper Corp. is a Canadian company listed on ASX via CHESS Depository Interests (CDIs, 1:1 ratio). All financials are in USD converted to AUD at 0.645 (approximate implied rate at data sourcing). Capstone does not file ASX Appendix 5B; financial data is sourced from Canadian MD&amp;A (Q1 CY2026, 29-Apr-2026). Its scale (200–230 kt Cu guidance) is substantially larger than other peers in this table.</t>
+          <t>Shown using accounting convention: positive = net debt position; parenthetical (negative) = net cash position. Figures from most recent Appendix 5B quarterly cashflow report (March 2026 quarter). USD-denominated debt (29M: US$120M RCF; CYM: US$27.3M Nebari) converted at 0.645 AUDUSD.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="14" customHeight="1">
       <c r="A22" s="30" t="inlineStr">
         <is>
-          <t>DVP note</t>
+          <t>Data pull date</t>
         </is>
       </c>
       <c r="B22" s="31" t="inlineStr">
         <is>
-          <t>Develop Global: 22 kt CuEq used per confirmed guidance. Woodlawn (NSW) Cu/Zn/Pb/Ag polymetallic. Formal FY2026 annual Cu/Zn guidance in kt has not been published as a specific annual target. Pb and Ag co-product guidance is not quantified and has been excluded from the CuEq calculation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="14" customHeight="1">
-      <c r="A23" s="30" t="inlineStr">
-        <is>
-          <t>Net (Cash)/Debt</t>
-        </is>
-      </c>
-      <c r="B23" s="31" t="inlineStr">
-        <is>
-          <t>Shown using accounting convention: positive = net debt position; parenthetical (negative) = net cash position. Figures from most recent Appendix 5B quarterly cashflow report (March 2026 quarter). USD-denominated debt (29M: US$120M RCF; CYM: US$27.3M Nebari; CSC: US$1,131.8M) converted at 0.645 AUDUSD.</t>
+          <t>Financial data and production guidance sourced from ASX announcements released April–May 2026 (reflecting March 2026 quarter). Share prices are live via IRESS RTD. Metal prices are live via IRESS RTD. This table refreshes automatically when IRESS is connected.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="14" customHeight="1">
-      <c r="A24" s="30" t="inlineStr">
-        <is>
-          <t>Data pull date</t>
-        </is>
-      </c>
-      <c r="B24" s="31" t="inlineStr">
-        <is>
-          <t>Financial data and production guidance sourced from ASX announcements released April–May 2026 (reflecting March 2026 quarter). Share prices are live via IRESS RTD. Metal prices are live via IRESS RTD. This table refreshes automatically when IRESS is connected.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="14" customHeight="1">
-      <c r="A26" s="32" t="inlineStr">
+      <c r="A24" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  LIVE METAL PRICE MONITOR  (via IRESS RTD)</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="33" t="inlineStr">
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="33" t="inlineStr">
         <is>
           <t>Cu (USD/t)</t>
         </is>
       </c>
-      <c r="B27" s="34">
+      <c r="B25" s="34">
         <f>@IRESSRtd("Quote","13","0","COPNY.ID")</f>
         <v/>
       </c>
-      <c r="C27" s="33" t="inlineStr">
+      <c r="C25" s="33" t="inlineStr">
         <is>
           <t>Au (USD/oz)</t>
         </is>
       </c>
-      <c r="D27" s="34">
+      <c r="D25" s="34">
         <f>@IRESSRtd("Quote","13","0","SPTGLD.IF")</f>
         <v/>
       </c>
-      <c r="E27" s="33" t="inlineStr">
+      <c r="E25" s="33" t="inlineStr">
         <is>
           <t>Ag (USD/oz)</t>
         </is>
       </c>
-      <c r="F27" s="35">
+      <c r="F25" s="35">
         <f>@IRESSRtd("Quote","13","0","SPTSLV.IF")</f>
         <v/>
       </c>
-      <c r="G27" s="33" t="inlineStr">
+      <c r="G25" s="33" t="inlineStr">
         <is>
           <t>Zn (USD/t)</t>
         </is>
       </c>
-      <c r="H27" s="34">
+      <c r="H25" s="34">
         <f>@IRESSRtd("Quote","13","0","ZINC.LME")</f>
         <v/>
       </c>
-      <c r="I27" s="33" t="inlineStr">
+      <c r="I25" s="33" t="inlineStr">
         <is>
           <t>Pb (USD/t)</t>
         </is>
       </c>
-      <c r="J27" s="36" t="inlineStr">
+      <c r="J25" s="36" t="inlineStr">
         <is>
           <t>AUD/USD</t>
         </is>
       </c>
-      <c r="K27" s="37">
+      <c r="K25" s="37">
         <f>@IRESSRtd("Quote","13","0","AUDUSD.FX")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="B23:K23"/>
+  <mergeCells count="11">
     <mergeCell ref="B22:K22"/>
-    <mergeCell ref="A26:K26"/>
     <mergeCell ref="B17:K17"/>
+    <mergeCell ref="A15:K15"/>
     <mergeCell ref="B18:K18"/>
     <mergeCell ref="B21:K21"/>
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A16:K16"/>
-    <mergeCell ref="B24:K24"/>
+    <mergeCell ref="A24:K24"/>
+    <mergeCell ref="B16:K16"/>
     <mergeCell ref="B20:K20"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="B19:K19"/>
@@ -1566,7 +1507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P52"/>
+  <dimension ref="A1:P50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2333,11 +2274,11 @@
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="46" t="inlineStr">
         <is>
-          <t>CSC</t>
+          <t>SFR</t>
         </is>
       </c>
       <c r="B23" s="58" t="n">
-        <v>215</v>
+        <v>0</v>
       </c>
       <c r="C23" s="58" t="n">
         <v>0</v>
@@ -2375,80 +2316,19 @@
         <f>SUM(G23:K23)</f>
         <v/>
       </c>
-      <c r="M23" s="58" t="n"/>
+      <c r="M23" s="58" t="n">
+        <v>157</v>
+      </c>
       <c r="N23" s="56">
         <f>IF(M23&gt;0,M23,L23)</f>
         <v/>
       </c>
       <c r="O23" s="47" t="inlineStr">
         <is>
-          <t>‡</t>
+          <t>†</t>
         </is>
       </c>
       <c r="P23" s="60" t="inlineStr">
-        <is>
-          <t>CY2026 production guidance (200–230 kt Cu); Q1 CY26 Results, 29-Apr-2026 (Pinto Valley AZ + Cozamin MX + Mantos Blancos CL + Mantoverde CL)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="42" t="inlineStr">
-        <is>
-          <t>SFR</t>
-        </is>
-      </c>
-      <c r="B24" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="C24" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="54">
-        <f>B24</f>
-        <v/>
-      </c>
-      <c r="H24" s="54">
-        <f>C24*$C$6/$C$5</f>
-        <v/>
-      </c>
-      <c r="I24" s="54">
-        <f>D24*$C$7/$C$5</f>
-        <v/>
-      </c>
-      <c r="J24" s="54">
-        <f>E24*$C$8/$C$5</f>
-        <v/>
-      </c>
-      <c r="K24" s="54">
-        <f>F24*$C$9/$C$5</f>
-        <v/>
-      </c>
-      <c r="L24" s="55">
-        <f>SUM(G24:K24)</f>
-        <v/>
-      </c>
-      <c r="M24" s="54" t="n">
-        <v>157</v>
-      </c>
-      <c r="N24" s="56">
-        <f>IF(M24&gt;0,M24,L24)</f>
-        <v/>
-      </c>
-      <c r="O24" s="43" t="inlineStr">
-        <is>
-          <t>†</t>
-        </is>
-      </c>
-      <c r="P24" s="57" t="inlineStr">
         <is>
           <t>FY2026 guidance (149–165 kt CuEq; guiding to lower half); Q3 FY26 Quarterly, 23-Apr-2026 (MATSA Spain + Motheo Botswana)</t>
         </is>
@@ -2621,371 +2501,319 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="46" t="inlineStr">
         <is>
-          <t>CSC</t>
+          <t>SFR</t>
         </is>
       </c>
       <c r="B38" s="49" t="inlineStr">
         <is>
-          <t>Capstone Copper Corp.</t>
+          <t>Sandfire Resources Limited</t>
         </is>
       </c>
       <c r="C38" s="58" t="n">
-        <v>763.7</v>
+        <v>466.6</v>
       </c>
       <c r="D38" s="60" t="inlineStr">
         <is>
-          <t>Q1 CY26 MD&amp;A (Canadian disclosure), 29-Apr-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="61" t="inlineStr">
+          <t>Q3 FY26 Quarterly (466.58M at 28-Mar-26), 23-Apr-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="14" customHeight="1">
+      <c r="A41" s="29" t="inlineStr">
+        <is>
+          <t>3B. NET CASH / (DEBT) — MOST RECENT QUARTERLY (APP 5B OR EQUIVALENT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="67" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B42" s="67" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C42" s="67" t="inlineStr">
+        <is>
+          <t>Cash (A$M)</t>
+        </is>
+      </c>
+      <c r="D42" s="67" t="inlineStr">
+        <is>
+          <t>Debt (A$M)</t>
+        </is>
+      </c>
+      <c r="E42" s="67" t="inlineStr">
+        <is>
+          <t>Net (Cash)/Debt (A$M)</t>
+        </is>
+      </c>
+      <c r="F42" s="67" t="inlineStr">
+        <is>
+          <t>Qtr End</t>
+        </is>
+      </c>
+      <c r="G42" s="67" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="61" t="inlineStr">
+        <is>
+          <t>AIS</t>
+        </is>
+      </c>
+      <c r="B43" s="62" t="inlineStr">
+        <is>
+          <t>Aeris Resources Limited</t>
+        </is>
+      </c>
+      <c r="C43" s="68" t="n">
+        <v>149.8</v>
+      </c>
+      <c r="D43" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="69" t="n">
+        <v>-149.8</v>
+      </c>
+      <c r="F43" s="70" t="inlineStr">
+        <is>
+          <t>31-Mar-26</t>
+        </is>
+      </c>
+      <c r="G43" s="64" t="inlineStr">
+        <is>
+          <t>Debt-free from Dec-2025. Tritton Cu mine (NSW) + Cracow Au mine (Qld).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="46" t="inlineStr">
+        <is>
+          <t>A1M</t>
+        </is>
+      </c>
+      <c r="B44" s="49" t="inlineStr">
+        <is>
+          <t>AIC Mines Limited</t>
+        </is>
+      </c>
+      <c r="C44" s="71" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="D44" s="71" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="E44" s="72" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="F44" s="47" t="inlineStr">
+        <is>
+          <t>31-Mar-26</t>
+        </is>
+      </c>
+      <c r="G44" s="60" t="inlineStr">
+        <is>
+          <t>Eloise Cu mine (NW Qld). Q3 cash depressed – A$8.3M concentrate on-site, shipped Apr. Trafigura facility A$45.3M.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="61" t="inlineStr">
+        <is>
+          <t>DVP</t>
+        </is>
+      </c>
+      <c r="B45" s="62" t="inlineStr">
+        <is>
+          <t>Develop Global Limited</t>
+        </is>
+      </c>
+      <c r="C45" s="68" t="n">
+        <v>180</v>
+      </c>
+      <c r="D45" s="68" t="n">
+        <v>158</v>
+      </c>
+      <c r="E45" s="69" t="n">
+        <v>-22</v>
+      </c>
+      <c r="F45" s="70" t="inlineStr">
+        <is>
+          <t>31-Mar-26</t>
+        </is>
+      </c>
+      <c r="G45" s="64" t="inlineStr">
+        <is>
+          <t>Woodlawn (NSW): Cu/Zn/Pb/Ag polymetallic. Also has large mining services division (&gt;A$50M/qtr revenue). 22 kt CuEq used per instruction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="46" t="inlineStr">
+        <is>
+          <t>29M</t>
+        </is>
+      </c>
+      <c r="B46" s="49" t="inlineStr">
+        <is>
+          <t>29Metals Limited</t>
+        </is>
+      </c>
+      <c r="C46" s="71" t="n">
+        <v>234</v>
+      </c>
+      <c r="D46" s="71" t="n">
+        <v>186</v>
+      </c>
+      <c r="E46" s="72" t="n">
+        <v>-48</v>
+      </c>
+      <c r="F46" s="47" t="inlineStr">
+        <is>
+          <t>31-Mar-26</t>
+        </is>
+      </c>
+      <c r="G46" s="60" t="inlineStr">
+        <is>
+          <t>Golden Grove (WA): Cu–Zn–Au–Ag. Zn guidance materially cut (Xantho Extended geotechnical event). Net cash A$48M per co. (31-Mar-26). US$120M RCF converted @ 0.645.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="61" t="inlineStr">
+        <is>
+          <t>AMI</t>
+        </is>
+      </c>
+      <c r="B47" s="62" t="inlineStr">
+        <is>
+          <t>Aurelia Metals Limited</t>
+        </is>
+      </c>
+      <c r="C47" s="68" t="n">
+        <v>94.7</v>
+      </c>
+      <c r="D47" s="68" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="E47" s="69" t="n">
+        <v>-86.10000000000001</v>
+      </c>
+      <c r="F47" s="70" t="inlineStr">
+        <is>
+          <t>31-Mar-26</t>
+        </is>
+      </c>
+      <c r="G47" s="64" t="inlineStr">
+        <is>
+          <t>Federation + Peak mines (Cobar, NSW). Au is primary revenue driver; Cu is minor co-product. A$150M facility committed but undrawn at 31-Mar-26.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="46" t="inlineStr">
+        <is>
+          <t>HGO</t>
+        </is>
+      </c>
+      <c r="B48" s="49" t="inlineStr">
+        <is>
+          <t>Hillgrove Resources Limited</t>
+        </is>
+      </c>
+      <c r="C48" s="71" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="D48" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="72" t="n">
+        <v>-25.2</v>
+      </c>
+      <c r="F48" s="47" t="inlineStr">
+        <is>
+          <t>31-Mar-26</t>
+        </is>
+      </c>
+      <c r="G48" s="60" t="inlineStr">
+        <is>
+          <t>Kanmantoo underground (SA). Pure copper producer (cathode + concentrate). Debt-free. Record Q1 CY26: 3,120 t Cu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="61" t="inlineStr">
+        <is>
+          <t>CYM</t>
+        </is>
+      </c>
+      <c r="B49" s="62" t="inlineStr">
+        <is>
+          <t>Cyprium Metals Limited</t>
+        </is>
+      </c>
+      <c r="C49" s="68" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="D49" s="68" t="n">
+        <v>42</v>
+      </c>
+      <c r="E49" s="69" t="n">
+        <v>-54.5</v>
+      </c>
+      <c r="F49" s="70" t="inlineStr">
+        <is>
+          <t>31-Mar-26</t>
+        </is>
+      </c>
+      <c r="G49" s="64" t="inlineStr">
+        <is>
+          <t>PRE-PRODUCTION. Nifty SX-EW cathode restart (Pilbara, WA). Phase 1 ~7 ktpa Cu; Phase 2 potential ~25 ktpa. US$27.3M Nebari facility ≈ A$42M @ 0.645.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="46" t="inlineStr">
         <is>
           <t>SFR</t>
         </is>
       </c>
-      <c r="B39" s="62" t="inlineStr">
+      <c r="B50" s="49" t="inlineStr">
         <is>
           <t>Sandfire Resources Limited</t>
         </is>
       </c>
-      <c r="C39" s="63" t="n">
-        <v>466.6</v>
-      </c>
-      <c r="D39" s="64" t="inlineStr">
-        <is>
-          <t>Q3 FY26 Quarterly (466.58M at 28-Mar-26), 23-Apr-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="14" customHeight="1">
-      <c r="A42" s="29" t="inlineStr">
-        <is>
-          <t>3B. NET CASH / (DEBT) — MOST RECENT QUARTERLY (APP 5B OR EQUIVALENT)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="67" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B43" s="67" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="C43" s="67" t="inlineStr">
-        <is>
-          <t>Cash (A$M)</t>
-        </is>
-      </c>
-      <c r="D43" s="67" t="inlineStr">
-        <is>
-          <t>Debt (A$M)</t>
-        </is>
-      </c>
-      <c r="E43" s="67" t="inlineStr">
-        <is>
-          <t>Net (Cash)/Debt (A$M)</t>
-        </is>
-      </c>
-      <c r="F43" s="67" t="inlineStr">
-        <is>
-          <t>Qtr End</t>
-        </is>
-      </c>
-      <c r="G43" s="67" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="61" t="inlineStr">
-        <is>
-          <t>AIS</t>
-        </is>
-      </c>
-      <c r="B44" s="62" t="inlineStr">
-        <is>
-          <t>Aeris Resources Limited</t>
-        </is>
-      </c>
-      <c r="C44" s="68" t="n">
-        <v>149.8</v>
-      </c>
-      <c r="D44" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="E44" s="69" t="n">
-        <v>-149.8</v>
-      </c>
-      <c r="F44" s="70" t="inlineStr">
+      <c r="C50" s="71" t="n">
+        <v>195.3</v>
+      </c>
+      <c r="D50" s="71" t="n">
+        <v>119.3</v>
+      </c>
+      <c r="E50" s="72" t="n">
+        <v>-76.00000000000001</v>
+      </c>
+      <c r="F50" s="47" t="inlineStr">
         <is>
           <t>31-Mar-26</t>
         </is>
       </c>
-      <c r="G44" s="64" t="inlineStr">
-        <is>
-          <t>Debt-free from Dec-2025. Tritton Cu mine (NSW) + Cracow Au mine (Qld).</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="46" t="inlineStr">
-        <is>
-          <t>A1M</t>
-        </is>
-      </c>
-      <c r="B45" s="49" t="inlineStr">
-        <is>
-          <t>AIC Mines Limited</t>
-        </is>
-      </c>
-      <c r="C45" s="71" t="n">
-        <v>31.1</v>
-      </c>
-      <c r="D45" s="71" t="n">
-        <v>45.3</v>
-      </c>
-      <c r="E45" s="72" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="F45" s="47" t="inlineStr">
-        <is>
-          <t>31-Mar-26</t>
-        </is>
-      </c>
-      <c r="G45" s="60" t="inlineStr">
-        <is>
-          <t>Eloise Cu mine (NW Qld). Q3 cash depressed – A$8.3M concentrate on-site, shipped Apr. Trafigura facility A$45.3M.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="61" t="inlineStr">
-        <is>
-          <t>DVP</t>
-        </is>
-      </c>
-      <c r="B46" s="62" t="inlineStr">
-        <is>
-          <t>Develop Global Limited</t>
-        </is>
-      </c>
-      <c r="C46" s="68" t="n">
-        <v>180</v>
-      </c>
-      <c r="D46" s="68" t="n">
-        <v>158</v>
-      </c>
-      <c r="E46" s="69" t="n">
-        <v>-22</v>
-      </c>
-      <c r="F46" s="70" t="inlineStr">
-        <is>
-          <t>31-Mar-26</t>
-        </is>
-      </c>
-      <c r="G46" s="64" t="inlineStr">
-        <is>
-          <t>Woodlawn (NSW): Cu/Zn/Pb/Ag polymetallic. Also has large mining services division (&gt;A$50M/qtr revenue). 22 kt CuEq used per instruction.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="46" t="inlineStr">
-        <is>
-          <t>29M</t>
-        </is>
-      </c>
-      <c r="B47" s="49" t="inlineStr">
-        <is>
-          <t>29Metals Limited</t>
-        </is>
-      </c>
-      <c r="C47" s="71" t="n">
-        <v>234</v>
-      </c>
-      <c r="D47" s="71" t="n">
-        <v>186</v>
-      </c>
-      <c r="E47" s="72" t="n">
-        <v>-48</v>
-      </c>
-      <c r="F47" s="47" t="inlineStr">
-        <is>
-          <t>31-Mar-26</t>
-        </is>
-      </c>
-      <c r="G47" s="60" t="inlineStr">
-        <is>
-          <t>Golden Grove (WA): Cu–Zn–Au–Ag. Zn guidance materially cut (Xantho Extended geotechnical event). Net cash A$48M per co. (31-Mar-26). US$120M RCF converted @ 0.645.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="61" t="inlineStr">
-        <is>
-          <t>AMI</t>
-        </is>
-      </c>
-      <c r="B48" s="62" t="inlineStr">
-        <is>
-          <t>Aurelia Metals Limited</t>
-        </is>
-      </c>
-      <c r="C48" s="68" t="n">
-        <v>94.7</v>
-      </c>
-      <c r="D48" s="68" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="E48" s="69" t="n">
-        <v>-86.10000000000001</v>
-      </c>
-      <c r="F48" s="70" t="inlineStr">
-        <is>
-          <t>31-Mar-26</t>
-        </is>
-      </c>
-      <c r="G48" s="64" t="inlineStr">
-        <is>
-          <t>Federation + Peak mines (Cobar, NSW). Au is primary revenue driver; Cu is minor co-product. A$150M facility committed but undrawn at 31-Mar-26.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="46" t="inlineStr">
-        <is>
-          <t>HGO</t>
-        </is>
-      </c>
-      <c r="B49" s="49" t="inlineStr">
-        <is>
-          <t>Hillgrove Resources Limited</t>
-        </is>
-      </c>
-      <c r="C49" s="71" t="n">
-        <v>25.2</v>
-      </c>
-      <c r="D49" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="E49" s="72" t="n">
-        <v>-25.2</v>
-      </c>
-      <c r="F49" s="47" t="inlineStr">
-        <is>
-          <t>31-Mar-26</t>
-        </is>
-      </c>
-      <c r="G49" s="60" t="inlineStr">
-        <is>
-          <t>Kanmantoo underground (SA). Pure copper producer (cathode + concentrate). Debt-free. Record Q1 CY26: 3,120 t Cu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="61" t="inlineStr">
-        <is>
-          <t>CYM</t>
-        </is>
-      </c>
-      <c r="B50" s="62" t="inlineStr">
-        <is>
-          <t>Cyprium Metals Limited</t>
-        </is>
-      </c>
-      <c r="C50" s="68" t="n">
-        <v>96.5</v>
-      </c>
-      <c r="D50" s="68" t="n">
-        <v>42</v>
-      </c>
-      <c r="E50" s="69" t="n">
-        <v>-54.5</v>
-      </c>
-      <c r="F50" s="70" t="inlineStr">
-        <is>
-          <t>31-Mar-26</t>
-        </is>
-      </c>
-      <c r="G50" s="64" t="inlineStr">
-        <is>
-          <t>PRE-PRODUCTION. Nifty SX-EW cathode restart (Pilbara, WA). Phase 1 ~7 ktpa Cu; Phase 2 potential ~25 ktpa. US$27.3M Nebari facility ≈ A$42M @ 0.645.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="46" t="inlineStr">
-        <is>
-          <t>CSC</t>
-        </is>
-      </c>
-      <c r="B51" s="49" t="inlineStr">
-        <is>
-          <t>Capstone Copper Corp.</t>
-        </is>
-      </c>
-      <c r="C51" s="71" t="n">
-        <v>611</v>
-      </c>
-      <c r="D51" s="71" t="n">
-        <v>1754</v>
-      </c>
-      <c r="E51" s="72" t="n">
-        <v>1143</v>
-      </c>
-      <c r="F51" s="47" t="inlineStr">
-        <is>
-          <t>31-Mar-26</t>
-        </is>
-      </c>
-      <c r="G51" s="60" t="inlineStr">
-        <is>
-          <t>Canadian co. / ASX CDI (1:1). All financials in USD, converted @ 0.645 AUDUSD. Files Canadian MD&amp;A (not App 5B). Co-products (Ag, Au, Mo) add incremental CuEq – not quantified here.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="61" t="inlineStr">
-        <is>
-          <t>SFR</t>
-        </is>
-      </c>
-      <c r="B52" s="62" t="inlineStr">
-        <is>
-          <t>Sandfire Resources Limited</t>
-        </is>
-      </c>
-      <c r="C52" s="68" t="n">
-        <v>195.3</v>
-      </c>
-      <c r="D52" s="68" t="n">
-        <v>119.3</v>
-      </c>
-      <c r="E52" s="69" t="n">
-        <v>-76.00000000000001</v>
-      </c>
-      <c r="F52" s="70" t="inlineStr">
-        <is>
-          <t>31-Mar-26</t>
-        </is>
-      </c>
-      <c r="G52" s="64" t="inlineStr">
+      <c r="G50" s="60" t="inlineStr">
         <is>
           <t>Company-disclosed CuEq. MATSA: Cu/Zn/Pb/Ag polymetallic. Motheo: copper only. Net cash A$76M per co. (31-Mar-26).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="17">
     <mergeCell ref="D38:F38"/>
     <mergeCell ref="A28:P28"/>
-    <mergeCell ref="A42:P42"/>
     <mergeCell ref="A13:P13"/>
     <mergeCell ref="A14:P14"/>
     <mergeCell ref="D37:F37"/>
@@ -2996,10 +2824,10 @@
     <mergeCell ref="D36:F36"/>
     <mergeCell ref="A3:P3"/>
     <mergeCell ref="A30:P30"/>
-    <mergeCell ref="D39:F39"/>
     <mergeCell ref="A29:P29"/>
     <mergeCell ref="D33:F33"/>
     <mergeCell ref="D34:F34"/>
+    <mergeCell ref="A41:P41"/>
     <mergeCell ref="A2:P2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>